<commit_message>
fix: recreate XLSX template with headers in row 1 col A - SheetJS was reading title row as headers causing import failure
</commit_message>
<xml_diff>
--- a/public/templates/modelo_contatos.xlsx
+++ b/public/templates/modelo_contatos.xlsx
@@ -19,7 +19,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="6">
+  <fonts count="4">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -28,33 +28,22 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <name val="Noto Sans CJK SC"/>
-      <color rgb="001B2A4A"/>
-      <sz val="16"/>
-    </font>
-    <font>
-      <name val="Noto Sans CJK SC"/>
+      <b val="1"/>
       <color rgb="00FFFFFF"/>
       <sz val="11"/>
     </font>
     <font>
-      <name val="Noto Sans CJK SC"/>
-      <i val="1"/>
-      <color rgb="008C8A84"/>
-      <sz val="9"/>
+      <b val="1"/>
+      <color rgb="001F4E79"/>
+      <sz val="14"/>
     </font>
     <font>
-      <name val="Noto Sans CJK SC"/>
-      <color rgb="0037352F"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <name val="Consolas"/>
-      <color rgb="001B2A4A"/>
+      <b val="1"/>
+      <color rgb="001F4E79"/>
       <sz val="11"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
@@ -63,17 +52,14 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="001B2A4A"/>
+        <fgColor rgb="001F4E79"/>
+        <bgColor rgb="001F4E79"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFFFFF"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00F7F7F5"/>
+        <fgColor rgb="00EBF5FB"/>
+        <bgColor rgb="00EBF5FB"/>
       </patternFill>
     </fill>
   </fills>
@@ -86,9 +72,10 @@
       <diagonal/>
     </border>
     <border>
-      <bottom style="thin">
-        <color rgb="00E9E9E8"/>
-      </bottom>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
     </border>
   </borders>
   <cellStyleXfs count="1">
@@ -96,17 +83,13 @@
   </cellStyleXfs>
   <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -472,261 +455,171 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:F19"/>
+  <dimension ref="A1:E6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="3" customWidth="1" min="1" max="1"/>
-    <col width="22" customWidth="1" min="2" max="2"/>
-    <col width="22" customWidth="1" min="3" max="3"/>
-    <col width="20" customWidth="1" min="4" max="4"/>
-    <col width="18" customWidth="1" min="5" max="5"/>
-    <col width="18" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="15" customWidth="1" min="4" max="4"/>
+    <col width="15" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
-    <row r="1" ht="15" customHeight="1"/>
-    <row r="2" ht="32" customHeight="1">
-      <c r="B2" s="1" t="inlineStr">
-        <is>
-          <t>Modelo de Contatos — OctupusZap</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="30" customHeight="1">
-      <c r="B3" s="2" t="inlineStr">
-        <is>
-          <t>Preencha os dados abaixo e importe no sistema. Coluna Telefone é obrigatória. Adicione mais colunas se quiser — elas viram variáveis {{coluna}} automaticamente!</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="28" customHeight="1">
-      <c r="B4" s="3" t="inlineStr">
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Empresa</t>
         </is>
       </c>
-      <c r="C4" s="3" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Nome</t>
         </is>
       </c>
-      <c r="D4" s="3" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Telefone</t>
         </is>
       </c>
-      <c r="E4" s="3" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Vendedor</t>
         </is>
       </c>
-      <c r="F4" s="3" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Nota</t>
         </is>
       </c>
     </row>
-    <row r="5" ht="22" customHeight="1">
-      <c r="B5" s="4" t="inlineStr">
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
         <is>
           <t>Tech Corp</t>
         </is>
       </c>
-      <c r="C5" s="4" t="inlineStr">
+      <c r="B2" s="2" t="inlineStr">
         <is>
           <t>João Silva</t>
         </is>
       </c>
-      <c r="D5" s="4" t="inlineStr">
+      <c r="C2" s="2" t="inlineStr">
         <is>
           <t>11999990001</t>
         </is>
       </c>
-      <c r="E5" s="4" t="inlineStr">
+      <c r="D2" s="2" t="inlineStr">
         <is>
           <t>Renato</t>
         </is>
       </c>
-      <c r="F5" s="4" t="inlineStr">
+      <c r="E2" s="2" t="inlineStr">
         <is>
           <t>VIP</t>
         </is>
       </c>
     </row>
-    <row r="6" ht="22" customHeight="1">
-      <c r="B6" s="5" t="inlineStr">
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
         <is>
           <t>Info Ltda</t>
         </is>
       </c>
-      <c r="C6" s="5" t="inlineStr">
+      <c r="B3" s="3" t="inlineStr">
         <is>
           <t>Maria Santos</t>
         </is>
       </c>
-      <c r="D6" s="5" t="inlineStr">
+      <c r="C3" s="3" t="inlineStr">
         <is>
           <t>21988880002</t>
         </is>
       </c>
-      <c r="E6" s="5" t="inlineStr">
+      <c r="D3" s="3" t="inlineStr">
         <is>
           <t>Carlos</t>
         </is>
       </c>
-      <c r="F6" s="5" t="inlineStr"/>
-    </row>
-    <row r="7" ht="22" customHeight="1">
-      <c r="B7" s="4" t="inlineStr">
+      <c r="E3" s="3" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
         <is>
           <t>Digital Inc</t>
         </is>
       </c>
-      <c r="C7" s="4" t="inlineStr">
+      <c r="B4" s="2" t="inlineStr">
         <is>
           <t>Pedro Lima</t>
         </is>
       </c>
-      <c r="D7" s="4" t="inlineStr">
+      <c r="C4" s="2" t="inlineStr">
         <is>
           <t>31977770003</t>
         </is>
       </c>
-      <c r="E7" s="4" t="inlineStr">
+      <c r="D4" s="2" t="inlineStr">
         <is>
           <t>Ana</t>
         </is>
       </c>
-      <c r="F7" s="4" t="inlineStr">
+      <c r="E4" s="2" t="inlineStr">
         <is>
           <t>Premium</t>
         </is>
       </c>
     </row>
-    <row r="8" ht="22" customHeight="1">
-      <c r="B8" s="5" t="inlineStr">
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
         <is>
           <t>Mega Sistemas</t>
         </is>
       </c>
-      <c r="C8" s="5" t="inlineStr">
+      <c r="B5" s="3" t="inlineStr">
         <is>
           <t>Carla Oliveira</t>
         </is>
       </c>
-      <c r="D8" s="5" t="inlineStr">
+      <c r="C5" s="3" t="inlineStr">
         <is>
           <t>41966660004</t>
         </is>
       </c>
-      <c r="E8" s="5" t="inlineStr">
+      <c r="D5" s="3" t="inlineStr">
         <is>
           <t>Renato</t>
         </is>
       </c>
-      <c r="F8" s="5" t="inlineStr"/>
-    </row>
-    <row r="9" ht="22" customHeight="1">
-      <c r="B9" s="4" t="inlineStr">
+      <c r="E5" s="3" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
         <is>
           <t>Alpha Tech</t>
         </is>
       </c>
-      <c r="C9" s="4" t="inlineStr">
+      <c r="B6" s="2" t="inlineStr">
         <is>
           <t>Lucas Ferreira</t>
         </is>
       </c>
-      <c r="D9" s="4" t="inlineStr">
+      <c r="C6" s="2" t="inlineStr">
         <is>
           <t>51955550005</t>
         </is>
       </c>
-      <c r="E9" s="4" t="inlineStr">
+      <c r="D6" s="2" t="inlineStr">
         <is>
           <t>Carlos</t>
         </is>
       </c>
-      <c r="F9" s="4" t="inlineStr">
+      <c r="E6" s="2" t="inlineStr">
         <is>
           <t>Prioridade</t>
         </is>
       </c>
     </row>
-    <row r="10" ht="22" customHeight="1">
-      <c r="B10" s="5" t="n"/>
-      <c r="C10" s="5" t="n"/>
-      <c r="D10" s="5" t="n"/>
-      <c r="E10" s="5" t="n"/>
-      <c r="F10" s="5" t="n"/>
-    </row>
-    <row r="11" ht="22" customHeight="1">
-      <c r="B11" s="4" t="n"/>
-      <c r="C11" s="4" t="n"/>
-      <c r="D11" s="4" t="n"/>
-      <c r="E11" s="4" t="n"/>
-      <c r="F11" s="4" t="n"/>
-    </row>
-    <row r="12" ht="22" customHeight="1">
-      <c r="B12" s="5" t="n"/>
-      <c r="C12" s="5" t="n"/>
-      <c r="D12" s="5" t="n"/>
-      <c r="E12" s="5" t="n"/>
-      <c r="F12" s="5" t="n"/>
-    </row>
-    <row r="13" ht="22" customHeight="1">
-      <c r="B13" s="4" t="n"/>
-      <c r="C13" s="4" t="n"/>
-      <c r="D13" s="4" t="n"/>
-      <c r="E13" s="4" t="n"/>
-      <c r="F13" s="4" t="n"/>
-    </row>
-    <row r="14" ht="22" customHeight="1">
-      <c r="B14" s="5" t="n"/>
-      <c r="C14" s="5" t="n"/>
-      <c r="D14" s="5" t="n"/>
-      <c r="E14" s="5" t="n"/>
-      <c r="F14" s="5" t="n"/>
-    </row>
-    <row r="15" ht="22" customHeight="1">
-      <c r="B15" s="4" t="n"/>
-      <c r="C15" s="4" t="n"/>
-      <c r="D15" s="4" t="n"/>
-      <c r="E15" s="4" t="n"/>
-      <c r="F15" s="4" t="n"/>
-    </row>
-    <row r="16" ht="22" customHeight="1">
-      <c r="B16" s="5" t="n"/>
-      <c r="C16" s="5" t="n"/>
-      <c r="D16" s="5" t="n"/>
-      <c r="E16" s="5" t="n"/>
-      <c r="F16" s="5" t="n"/>
-    </row>
-    <row r="17" ht="22" customHeight="1">
-      <c r="B17" s="4" t="n"/>
-      <c r="C17" s="4" t="n"/>
-      <c r="D17" s="4" t="n"/>
-      <c r="E17" s="4" t="n"/>
-      <c r="F17" s="4" t="n"/>
-    </row>
-    <row r="18" ht="22" customHeight="1">
-      <c r="B18" s="5" t="n"/>
-      <c r="C18" s="5" t="n"/>
-      <c r="D18" s="5" t="n"/>
-      <c r="E18" s="5" t="n"/>
-      <c r="F18" s="5" t="n"/>
-    </row>
-    <row r="19" ht="22" customHeight="1">
-      <c r="B19" s="4" t="n"/>
-      <c r="C19" s="4" t="n"/>
-      <c r="D19" s="4" t="n"/>
-      <c r="E19" s="4" t="n"/>
-      <c r="F19" s="4" t="n"/>
-    </row>
   </sheetData>
-  <mergeCells count="2">
-    <mergeCell ref="B2:F2"/>
-    <mergeCell ref="B3:F3"/>
-  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -737,164 +630,120 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:D12"/>
+  <dimension ref="A1:A17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="3" customWidth="1" min="1" max="1"/>
-    <col width="8" customWidth="1" min="2" max="2"/>
-    <col width="48" customWidth="1" min="3" max="3"/>
-    <col width="40" customWidth="1" min="4" max="4"/>
+    <col width="70" customWidth="1" min="1" max="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="15" customHeight="1"/>
-    <row r="2" ht="32" customHeight="1">
-      <c r="B2" s="1" t="inlineStr">
-        <is>
-          <t>Como Usar Este Arquivo</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="8" customHeight="1"/>
-    <row r="5" ht="28" customHeight="1">
-      <c r="B5" s="3" t="inlineStr">
-        <is>
-          <t>Passo</t>
-        </is>
-      </c>
-      <c r="C5" s="3" t="inlineStr">
-        <is>
-          <t>Instrução</t>
-        </is>
-      </c>
-      <c r="D5" s="3" t="inlineStr">
-        <is>
-          <t>Exemplo</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="22" customHeight="1">
-      <c r="B6" s="5" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="C6" s="5" t="inlineStr">
-        <is>
-          <t>Preencha a aba 'Contatos' com os dados dos clientes</t>
-        </is>
-      </c>
-      <c r="D6" s="5" t="inlineStr">
-        <is>
-          <t>Empresa: Tech Corp, Nome: João Silva</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="22" customHeight="1">
-      <c r="B7" s="4" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="C7" s="4" t="inlineStr">
-        <is>
-          <t>A coluna Telefone é obrigatória (com DDD)</t>
-        </is>
-      </c>
-      <c r="D7" s="4" t="inlineStr">
-        <is>
-          <t>11999990001 ou 5511999990001</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="22" customHeight="1">
-      <c r="B8" s="5" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="C8" s="5" t="inlineStr">
-        <is>
-          <t>As colunas Nome e Empresa são recomendadas</t>
-        </is>
-      </c>
-      <c r="D8" s="5" t="inlineStr">
-        <is>
-          <t>Usadas como {{nome}} e {{empresa}} nas mensagens</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="22" customHeight="1">
-      <c r="B9" s="4" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="C9" s="4" t="inlineStr">
-        <is>
-          <t>Adicione quantas colunas quiser após a coluna F</t>
-        </is>
-      </c>
-      <c r="D9" s="4" t="inlineStr">
-        <is>
-          <t>Ex: Cidade, Segmento, Produto, Observação</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="22" customHeight="1">
-      <c r="B10" s="5" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
-      </c>
-      <c r="C10" s="5" t="inlineStr">
-        <is>
-          <t>Cada coluna vira uma variável {{nome_da_coluna}}</t>
-        </is>
-      </c>
-      <c r="D10" s="5" t="inlineStr">
-        <is>
-          <t>Coluna 'Nota' → use {{nota}} na mensagem</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="22" customHeight="1">
-      <c r="B11" s="4" t="inlineStr">
-        <is>
-          <t>6</t>
-        </is>
-      </c>
-      <c r="C11" s="4" t="inlineStr">
-        <is>
-          <t>Salve o arquivo e importe no OctupusZap</t>
-        </is>
-      </c>
-      <c r="D11" s="4" t="inlineStr">
-        <is>
-          <t>Menu Contatos → Importar Planilha</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="22" customHeight="1">
-      <c r="B12" s="5" t="inlineStr">
-        <is>
-          <t>7</t>
-        </is>
-      </c>
-      <c r="C12" s="5" t="inlineStr">
-        <is>
-          <t>Na campanha, as variáveis aparecem como chips clicáveis</t>
-        </is>
-      </c>
-      <c r="D12" s="5" t="inlineStr">
-        <is>
-          <t>Selecione a lista de contatos primeiro</t>
+    <row r="1">
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t>Instruções de Uso — Planilha Modelo OctupusZap</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>1. PREENCHA a aba 'Contatos' com seus dados</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2. A coluna TELEFONE é obrigatória — é o número que receberá o WhatsApp</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>3. Adicione QUANTAS COLUNAS quiser (empresa, cidade, produto, etc.)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>4. Cada coluna vira uma variável automática: {{nome}}, {{empresa}}, {{cidade}}</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>5. Use essas variáveis no texto da mensagem para personalizar</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Exemplos de variáveis:</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  {{nome}} → Nome do contato</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  {{telefone}} → Telefone do contato</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  {{empresa}} → Empresa do contato</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  {{vendedor}} → Vendedor responsável</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  {{nota}} → Qualquer campo extra que você adicionar</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Formatos aceitos: CSV, XLSX, XLS, ODS</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Telefone: pode ser com ou sem código do país (55)</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="B2:C2"/>
-  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -905,147 +754,117 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:D11"/>
+  <dimension ref="A1:C6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="3" customWidth="1" min="1" max="1"/>
-    <col width="24" customWidth="1" min="2" max="2"/>
-    <col width="40" customWidth="1" min="3" max="3"/>
-    <col width="44" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="25" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
-    <row r="1" ht="15" customHeight="1"/>
-    <row r="2" ht="32" customHeight="1">
-      <c r="B2" s="1" t="inlineStr">
-        <is>
-          <t>Variáveis Disponíveis nas Mensagens</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="8" customHeight="1"/>
-    <row r="5" ht="28" customHeight="1">
-      <c r="B5" s="3" t="inlineStr">
+    <row r="1">
+      <c r="A1" s="5" t="inlineStr">
         <is>
           <t>Variável</t>
         </is>
       </c>
-      <c r="C5" s="3" t="inlineStr">
+      <c r="B1" s="5" t="inlineStr">
         <is>
           <t>Origem</t>
         </is>
       </c>
-      <c r="D5" s="3" t="inlineStr">
-        <is>
-          <t>Exemplo de Uso</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="22" customHeight="1">
-      <c r="B6" s="5" t="inlineStr">
+      <c r="C1" s="5" t="inlineStr">
+        <is>
+          <t>Exemplo</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
         <is>
           <t>{{nome}}</t>
         </is>
       </c>
-      <c r="C6" s="5" t="inlineStr">
-        <is>
-          <t>Coluna Nome da planilha</t>
-        </is>
-      </c>
-      <c r="D6" s="5" t="inlineStr">
-        <is>
-          <t>Olá {{nome}}, tudo bem?</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="22" customHeight="1">
-      <c r="B7" s="4" t="inlineStr">
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Coluna Nome</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>João Silva</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
         <is>
           <t>{{telefone}}</t>
         </is>
       </c>
-      <c r="C7" s="4" t="inlineStr">
-        <is>
-          <t>Coluna Telefone da planilha</t>
-        </is>
-      </c>
-      <c r="D7" s="4" t="inlineStr">
-        <is>
-          <t>Este número é de {{nome}}?</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="22" customHeight="1">
-      <c r="B8" s="5" t="inlineStr">
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Coluna Telefone</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>11999990001</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
         <is>
           <t>{{empresa}}</t>
         </is>
       </c>
-      <c r="C8" s="5" t="inlineStr">
-        <is>
-          <t>Coluna Empresa da planilha</t>
-        </is>
-      </c>
-      <c r="D8" s="5" t="inlineStr">
-        <is>
-          <t>Sou da MTech, falo com compras da {{empresa}}?</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="22" customHeight="1">
-      <c r="B9" s="4" t="inlineStr">
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Coluna Empresa</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Tech Corp</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
         <is>
           <t>{{vendedor}}</t>
         </is>
       </c>
-      <c r="C9" s="4" t="inlineStr">
-        <is>
-          <t>Coluna Vendedor da planilha</t>
-        </is>
-      </c>
-      <c r="D9" s="4" t="inlineStr">
-        <is>
-          <t>Meu nome é {{vendedor}}, sou da MTech</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="22" customHeight="1">
-      <c r="B10" s="5" t="inlineStr">
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Coluna Vendedor</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Renato</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
         <is>
           <t>{{nota}}</t>
         </is>
       </c>
-      <c r="C10" s="5" t="inlineStr">
-        <is>
-          <t>Coluna Nota da planilha</t>
-        </is>
-      </c>
-      <c r="D10" s="5" t="inlineStr">
-        <is>
-          <t>Cliente {{nota}}: {{nome}}</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="22" customHeight="1">
-      <c r="B11" s="4" t="inlineStr">
-        <is>
-          <t>{{qualquer_coluna}}</t>
-        </is>
-      </c>
-      <c r="C11" s="4" t="inlineStr">
-        <is>
-          <t>Qualquer coluna que você adicionar</t>
-        </is>
-      </c>
-      <c r="D11" s="4" t="inlineStr">
-        <is>
-          <t>Basta criar a coluna e usar {{nome_da_coluna}}</t>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Coluna Nota</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>VIP</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="B2:C2"/>
-  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: emoji picker, preview scroll fix, WhatsApp column in contact template
</commit_message>
<xml_diff>
--- a/public/templates/modelo_contatos.xlsx
+++ b/public/templates/modelo_contatos.xlsx
@@ -8,8 +8,6 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Contatos" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instruções" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Variáveis" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -19,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="4">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -32,18 +30,8 @@
       <color rgb="00FFFFFF"/>
       <sz val="11"/>
     </font>
-    <font>
-      <b val="1"/>
-      <color rgb="001F4E79"/>
-      <sz val="14"/>
-    </font>
-    <font>
-      <b val="1"/>
-      <color rgb="001F4E79"/>
-      <sz val="11"/>
-    </font>
   </fonts>
-  <fills count="4">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
@@ -52,18 +40,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="001F4E79"/>
-        <bgColor rgb="001F4E79"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00EBF5FB"/>
-        <bgColor rgb="00EBF5FB"/>
+        <fgColor rgb="0010B981"/>
+        <bgColor rgb="0010B981"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -71,25 +53,15 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -455,14 +427,15 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E6"/>
+  <dimension ref="A1:F6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="18" customWidth="1" min="1" max="1"/>
-    <col width="20" customWidth="1" min="2" max="2"/>
-    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="15" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="13" customWidth="1" min="3" max="3"/>
     <col width="15" customWidth="1" min="4" max="4"/>
-    <col width="15" customWidth="1" min="5" max="5"/>
+    <col width="11" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -483,384 +456,169 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>Vendedor</t>
+          <t>WhatsApp</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Vendedora</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Nota</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr">
+      <c r="A2" t="inlineStr">
         <is>
           <t>Tech Corp</t>
         </is>
       </c>
-      <c r="B2" s="2" t="inlineStr">
+      <c r="B2" t="inlineStr">
         <is>
           <t>João Silva</t>
         </is>
       </c>
-      <c r="C2" s="2" t="inlineStr">
+      <c r="C2" t="inlineStr">
         <is>
           <t>11999990001</t>
         </is>
       </c>
-      <c r="D2" s="2" t="inlineStr">
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>5511999990001</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
         <is>
           <t>Renato</t>
         </is>
       </c>
-      <c r="E2" s="2" t="inlineStr">
+      <c r="F2" t="inlineStr">
         <is>
           <t>VIP</t>
         </is>
       </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="3" t="inlineStr">
-        <is>
-          <t>Info Ltda</t>
-        </is>
-      </c>
-      <c r="B3" s="3" t="inlineStr">
-        <is>
-          <t>Maria Santos</t>
-        </is>
-      </c>
-      <c r="C3" s="3" t="inlineStr">
-        <is>
-          <t>21988880002</t>
-        </is>
-      </c>
-      <c r="D3" s="3" t="inlineStr">
-        <is>
-          <t>Carlos</t>
-        </is>
-      </c>
-      <c r="E3" s="3" t="inlineStr"/>
-    </row>
-    <row r="4">
-      <c r="A4" s="2" t="inlineStr">
-        <is>
-          <t>Digital Inc</t>
-        </is>
-      </c>
-      <c r="B4" s="2" t="inlineStr">
-        <is>
-          <t>Pedro Lima</t>
-        </is>
-      </c>
-      <c r="C4" s="2" t="inlineStr">
-        <is>
-          <t>31977770003</t>
-        </is>
-      </c>
-      <c r="D4" s="2" t="inlineStr">
-        <is>
-          <t>Ana</t>
-        </is>
-      </c>
-      <c r="E4" s="2" t="inlineStr">
-        <is>
-          <t>Premium</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="3" t="inlineStr">
-        <is>
-          <t>Mega Sistemas</t>
-        </is>
-      </c>
-      <c r="B5" s="3" t="inlineStr">
-        <is>
-          <t>Carla Oliveira</t>
-        </is>
-      </c>
-      <c r="C5" s="3" t="inlineStr">
-        <is>
-          <t>41966660004</t>
-        </is>
-      </c>
-      <c r="D5" s="3" t="inlineStr">
-        <is>
-          <t>Renato</t>
-        </is>
-      </c>
-      <c r="E5" s="3" t="inlineStr"/>
-    </row>
-    <row r="6">
-      <c r="A6" s="2" t="inlineStr">
-        <is>
-          <t>Alpha Tech</t>
-        </is>
-      </c>
-      <c r="B6" s="2" t="inlineStr">
-        <is>
-          <t>Lucas Ferreira</t>
-        </is>
-      </c>
-      <c r="C6" s="2" t="inlineStr">
-        <is>
-          <t>51955550005</t>
-        </is>
-      </c>
-      <c r="D6" s="2" t="inlineStr">
-        <is>
-          <t>Carlos</t>
-        </is>
-      </c>
-      <c r="E6" s="2" t="inlineStr">
-        <is>
-          <t>Prioridade</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:A17"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="70" customWidth="1" min="1" max="1"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="4" t="inlineStr">
-        <is>
-          <t>Instruções de Uso — Planilha Modelo OctupusZap</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>1. PREENCHA a aba 'Contatos' com seus dados</t>
-        </is>
-      </c>
+          <t>Info Ltda</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Maria Santos</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>21988880002</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>5521988880002</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Carlos</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2. A coluna TELEFONE é obrigatória — é o número que receberá o WhatsApp</t>
+          <t>Digital Inc</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Pedro Lima</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>31977770003</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>5531977770003</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Ana</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Premium</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>3. Adicione QUANTAS COLUNAS quiser (empresa, cidade, produto, etc.)</t>
-        </is>
-      </c>
+          <t>Mega Sistemas</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Carla Oliveira</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>41966660004</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>5541966660004</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Renato</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>4. Cada coluna vira uma variável automática: {{nome}}, {{empresa}}, {{cidade}}</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>5. Use essas variáveis no texto da mensagem para personalizar</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr"/>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>Exemplos de variáveis:</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  {{nome}} → Nome do contato</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  {{telefone}} → Telefone do contato</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  {{empresa}} → Empresa do contato</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  {{vendedor}} → Vendedor responsável</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  {{nota}} → Qualquer campo extra que você adicionar</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr"/>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>Formatos aceitos: CSV, XLSX, XLS, ODS</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>Telefone: pode ser com ou sem código do país (55)</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:C6"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="18" customWidth="1" min="1" max="1"/>
-    <col width="20" customWidth="1" min="2" max="2"/>
-    <col width="25" customWidth="1" min="3" max="3"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="5" t="inlineStr">
-        <is>
-          <t>Variável</t>
-        </is>
-      </c>
-      <c r="B1" s="5" t="inlineStr">
-        <is>
-          <t>Origem</t>
-        </is>
-      </c>
-      <c r="C1" s="5" t="inlineStr">
-        <is>
-          <t>Exemplo</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>{{nome}}</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>Coluna Nome</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>João Silva</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>{{telefone}}</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>Coluna Telefone</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>11999990001</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>{{empresa}}</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Coluna Empresa</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>Tech Corp</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>{{vendedor}}</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>Coluna Vendedor</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>Renato</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>{{nota}}</t>
+          <t>Alpha Tech</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Coluna Nota</t>
+          <t>Lucas Ferreira</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>VIP</t>
+          <t>51955550005</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>5551955550005</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Carlos</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Prioridade</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: fixed contact fields, template header, duplicate campaign, save as template
- Standard contact fields always shown: Nome, Telefone, Codigo, Empresa, Vendedora, Whatsapp, Nota
- Template spreadsheet has correct 7-column header
- Add Contact dialog shows all 7 fields
- Edit Contact dialog shows all 7 fields
- Duplicate campaign button on campaign cards
- Save campaign as template button on campaign cards
- MessageTemplate.steps field for multi-step campaign templates
- DB migration for steps column
- No wa.me links needed - numbers are clickable in WhatsApp natively
</commit_message>
<xml_diff>
--- a/public/templates/modelo_contatos.xlsx
+++ b/public/templates/modelo_contatos.xlsx
@@ -397,12 +397,15 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D6"/>
+  <dimension ref="A1:G4"/>
   <cols>
-    <col min="1" max="1" width="20.83203125" customWidth="1"/>
-    <col min="2" max="2" width="18.83203125" customWidth="1"/>
-    <col min="3" max="3" width="18.83203125" customWidth="1"/>
-    <col min="4" max="4" width="15.83203125" customWidth="1"/>
+    <col min="1" max="1" width="25.83203125" customWidth="1"/>
+    <col min="2" max="2" width="20.83203125" customWidth="1"/>
+    <col min="3" max="3" width="15.83203125" customWidth="1"/>
+    <col min="4" max="4" width="25.83203125" customWidth="1"/>
+    <col min="5" max="5" width="20.83203125" customWidth="1"/>
+    <col min="6" max="6" width="20.83203125" customWidth="1"/>
+    <col min="7" max="7" width="30.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -410,13 +413,22 @@
         <v>Nome</v>
       </c>
       <c r="B1" t="str">
-        <v>WhatsApp</v>
+        <v>Telefone</v>
       </c>
       <c r="C1" t="str">
+        <v>Codigo</v>
+      </c>
+      <c r="D1" t="str">
         <v>Empresa</v>
       </c>
-      <c r="D1" t="str">
+      <c r="E1" t="str">
         <v>Vendedora</v>
+      </c>
+      <c r="F1" t="str">
+        <v>Whatsapp</v>
+      </c>
+      <c r="G1" t="str">
+        <v>Nota</v>
       </c>
     </row>
     <row r="2">
@@ -427,10 +439,19 @@
         <v>5511999990001</v>
       </c>
       <c r="C2" t="str">
+        <v>001</v>
+      </c>
+      <c r="D2" t="str">
         <v>Tech Corp</v>
       </c>
-      <c r="D2" t="str">
+      <c r="E2" t="str">
         <v>Ana</v>
+      </c>
+      <c r="F2" t="str">
+        <v>5511999990001</v>
+      </c>
+      <c r="G2" t="str">
+        <v/>
       </c>
     </row>
     <row r="3">
@@ -441,10 +462,19 @@
         <v>5521988880002</v>
       </c>
       <c r="C3" t="str">
+        <v>002</v>
+      </c>
+      <c r="D3" t="str">
         <v>Info Ltda</v>
       </c>
-      <c r="D3" t="str">
+      <c r="E3" t="str">
         <v>Carla</v>
+      </c>
+      <c r="F3" t="str">
+        <v>5521988880002</v>
+      </c>
+      <c r="G3" t="str">
+        <v/>
       </c>
     </row>
     <row r="4">
@@ -455,43 +485,24 @@
         <v>5531977770003</v>
       </c>
       <c r="C4" t="str">
+        <v>003</v>
+      </c>
+      <c r="D4" t="str">
         <v>Digital Inc</v>
       </c>
-      <c r="D4" t="str">
+      <c r="E4" t="str">
         <v>Fernanda</v>
       </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="str">
-        <v>Carla Oliveira</v>
-      </c>
-      <c r="B5" t="str">
-        <v>5541966660004</v>
-      </c>
-      <c r="C5" t="str">
-        <v>Mega Sistemas</v>
-      </c>
-      <c r="D5" t="str">
-        <v>Patricia</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="str">
-        <v>Lucas Ferreira</v>
-      </c>
-      <c r="B6" t="str">
-        <v>5551955550005</v>
-      </c>
-      <c r="C6" t="str">
-        <v>Alpha Tech</v>
-      </c>
-      <c r="D6" t="str">
-        <v>Renata</v>
+      <c r="F4" t="str">
+        <v>5531977770003</v>
+      </c>
+      <c r="G4" t="str">
+        <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D6"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G4"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>